<commit_message>
Package the current map for a single Coolify deploy.
One container serves the site and reads MotherDuck. Scoring stays a local job.
</commit_message>
<xml_diff>
--- a/docs/likelihood-brackets.xlsx
+++ b/docs/likelihood-brackets.xlsx
@@ -589,7 +589,7 @@
     <row r="3" ht="24" customHeight="1">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>5  Almost certain</t>
+          <t>5  Very high</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -619,7 +619,7 @@
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>4  Likely</t>
+          <t>4  High</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -649,7 +649,7 @@
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>3  Possible</t>
+          <t>3  Medium</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -679,7 +679,7 @@
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>2  Unlikely</t>
+          <t>2  Low</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -696,7 +696,7 @@
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>1  Rare</t>
+          <t>1  Very low</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">

</xml_diff>